<commit_message>
adds psychological state and time interval
</commit_message>
<xml_diff>
--- a/data/Capus_LHommeBicycle_1893/Capus_LHommeBicycle_1893.xlsx
+++ b/data/Capus_LHommeBicycle_1893/Capus_LHommeBicycle_1893.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mathilde\Desktop\Doctorat - 2025-2028\Pipeline\SFonto\data\Capus_LHommeBicycle_1893\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84BF3EA7-3754-4B19-9996-54F811C8604E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61CC6BE3-FFAB-440E-89FE-E2BCA8D18353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Work" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="427">
   <si>
     <t>Classe</t>
   </si>
@@ -521,16 +521,7 @@
     <t>has location</t>
   </si>
   <si>
-    <t>:Age_Marius_4yo</t>
-  </si>
-  <si>
-    <t>:Age_Marius_20yo</t>
-  </si>
-  <si>
     <t>Time_Interval</t>
-  </si>
-  <si>
-    <t>:type_age</t>
   </si>
   <si>
     <t>:type_institutional_location</t>
@@ -795,9 +786,6 @@
     <t>participant</t>
   </si>
   <si>
-    <t>temporal location</t>
-  </si>
-  <si>
     <t>P16 used specific object</t>
   </si>
   <si>
@@ -1051,10 +1039,6 @@
     <t>:temporally-overlaps :Event_melancholy</t>
   </si>
   <si>
-    <t>:temporally-overlaps :Event_meet_Marius_Princess,
-:temporally-overlaps :Event_wedding</t>
-  </si>
-  <si>
     <t>Marius is from Provence</t>
   </si>
   <si>
@@ -1331,6 +1315,21 @@
   </si>
   <si>
     <t>:KnowsByReputation_Role</t>
+  </si>
+  <si>
+    <t>state of</t>
+  </si>
+  <si>
+    <t>:follows :Event_meet_Marius_Princess</t>
+  </si>
+  <si>
+    <t>:Time_Marius_4yo</t>
+  </si>
+  <si>
+    <t>:Time_Marius_20yo</t>
+  </si>
+  <si>
+    <t>temporal location / duration</t>
   </si>
 </sst>
 </file>
@@ -1529,7 +1528,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1642,6 +1641,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1649,8 +1653,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2018,13 +2021,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="51" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
@@ -2048,10 +2051,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>5</v>
@@ -2065,10 +2068,10 @@
       <c r="B4" s="3"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -2109,10 +2112,10 @@
       <c r="B8" s="3"/>
       <c r="C8" s="13"/>
       <c r="D8" s="3" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="41" customFormat="1" x14ac:dyDescent="0.3">
@@ -2120,10 +2123,10 @@
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
@@ -2131,7 +2134,7 @@
       <c r="B10" s="3"/>
       <c r="C10" s="13"/>
       <c r="D10" s="3" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>136</v>
@@ -2142,10 +2145,10 @@
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="21" customFormat="1" x14ac:dyDescent="0.3">
@@ -2153,7 +2156,7 @@
       <c r="B12" s="3"/>
       <c r="C12" s="13"/>
       <c r="D12" s="13" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E12" s="13" t="s">
         <v>79</v>
@@ -2164,7 +2167,7 @@
       <c r="B13" s="33"/>
       <c r="C13" s="33"/>
       <c r="D13" s="33" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E13" s="33" t="s">
         <v>78</v>
@@ -2175,7 +2178,7 @@
       <c r="B14" s="3"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="E14" s="13" t="s">
         <v>54</v>
@@ -2186,7 +2189,7 @@
       <c r="B15" s="33"/>
       <c r="C15" s="33"/>
       <c r="D15" s="20" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="E15" s="20" t="s">
         <v>56</v>
@@ -2197,7 +2200,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>61</v>
@@ -2206,7 +2209,7 @@
         <v>10</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -2272,13 +2275,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="51" t="s">
         <v>118</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -2291,10 +2294,10 @@
         <v>119</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2308,10 +2311,10 @@
         <v>55</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2319,10 +2322,10 @@
       <c r="B4" s="20"/>
       <c r="C4" s="20"/>
       <c r="D4" s="20" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2330,10 +2333,10 @@
       <c r="B5" s="22"/>
       <c r="C5" s="22"/>
       <c r="D5" s="22" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2341,10 +2344,10 @@
       <c r="B6" s="20"/>
       <c r="C6" s="20"/>
       <c r="D6" s="20" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2352,10 +2355,10 @@
       <c r="B7" s="22"/>
       <c r="C7" s="22"/>
       <c r="D7" s="22" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2363,10 +2366,10 @@
       <c r="B8" s="20"/>
       <c r="C8" s="20"/>
       <c r="D8" s="20" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2374,10 +2377,10 @@
       <c r="B9" s="22"/>
       <c r="C9" s="22"/>
       <c r="D9" s="22" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2385,10 +2388,10 @@
       <c r="B10" s="20"/>
       <c r="C10" s="20"/>
       <c r="D10" s="20" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2396,10 +2399,10 @@
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
       <c r="D11" s="22" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2407,10 +2410,10 @@
       <c r="B12" s="20"/>
       <c r="C12" s="20"/>
       <c r="D12" s="20" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="E12" s="20" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2418,10 +2421,10 @@
       <c r="B13" s="22"/>
       <c r="C13" s="22"/>
       <c r="D13" s="22" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2429,10 +2432,10 @@
       <c r="B14" s="20"/>
       <c r="C14" s="20"/>
       <c r="D14" s="20" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2440,10 +2443,10 @@
       <c r="B15" s="22"/>
       <c r="C15" s="22"/>
       <c r="D15" s="22" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2451,10 +2454,10 @@
       <c r="B16" s="20"/>
       <c r="C16" s="20"/>
       <c r="D16" s="20" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2462,10 +2465,10 @@
       <c r="B17" s="22"/>
       <c r="C17" s="22"/>
       <c r="D17" s="22" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2473,10 +2476,10 @@
       <c r="B18" s="20"/>
       <c r="C18" s="20"/>
       <c r="D18" s="20" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="E18" s="20" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2484,10 +2487,10 @@
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
       <c r="D19" s="22" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2495,10 +2498,10 @@
       <c r="B20" s="20"/>
       <c r="C20" s="20"/>
       <c r="D20" s="20" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2506,10 +2509,10 @@
       <c r="B21" s="22"/>
       <c r="C21" s="22"/>
       <c r="D21" s="22" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2517,10 +2520,10 @@
       <c r="B22" s="20"/>
       <c r="C22" s="20"/>
       <c r="D22" s="20" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E22" s="20" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2528,10 +2531,10 @@
       <c r="B23" s="22"/>
       <c r="C23" s="22"/>
       <c r="D23" s="22" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2539,10 +2542,10 @@
       <c r="B24" s="20"/>
       <c r="C24" s="20"/>
       <c r="D24" s="20" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="E24" s="20" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="16" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2550,10 +2553,10 @@
       <c r="B25" s="22"/>
       <c r="C25" s="22"/>
       <c r="D25" s="22" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2567,10 +2570,10 @@
         <v>57</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="E26" s="20" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
@@ -2578,10 +2581,10 @@
       <c r="B27" s="22"/>
       <c r="C27" s="22"/>
       <c r="D27" s="22" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
@@ -2589,10 +2592,10 @@
       <c r="B28" s="20"/>
       <c r="C28" s="20"/>
       <c r="D28" s="20" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="E28" s="20" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
@@ -2600,10 +2603,10 @@
       <c r="B29" s="22"/>
       <c r="C29" s="22"/>
       <c r="D29" s="22" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -2611,10 +2614,10 @@
       <c r="B30" s="20"/>
       <c r="C30" s="20"/>
       <c r="D30" s="20" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="E30" s="20" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
@@ -2622,10 +2625,10 @@
       <c r="B31" s="22"/>
       <c r="C31" s="22"/>
       <c r="D31" s="22" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
@@ -2633,10 +2636,10 @@
       <c r="B32" s="20"/>
       <c r="C32" s="20"/>
       <c r="D32" s="20" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="E32" s="20" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
@@ -2644,10 +2647,10 @@
       <c r="B33" s="22"/>
       <c r="C33" s="22"/>
       <c r="D33" s="22" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
@@ -2655,10 +2658,10 @@
       <c r="B34" s="20"/>
       <c r="C34" s="20"/>
       <c r="D34" s="20" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="E34" s="20" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
@@ -2666,10 +2669,10 @@
       <c r="B35" s="22"/>
       <c r="C35" s="22"/>
       <c r="D35" s="22" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
@@ -2677,10 +2680,10 @@
       <c r="B36" s="20"/>
       <c r="C36" s="20"/>
       <c r="D36" s="20" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="E36" s="20" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
@@ -2688,10 +2691,10 @@
       <c r="B37" s="22"/>
       <c r="C37" s="22"/>
       <c r="D37" s="22" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
@@ -2699,10 +2702,10 @@
       <c r="B38" s="20"/>
       <c r="C38" s="20"/>
       <c r="D38" s="20" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="E38" s="20" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
@@ -2710,10 +2713,10 @@
       <c r="B39" s="22"/>
       <c r="C39" s="22"/>
       <c r="D39" s="22" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="E39" s="22" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
@@ -2721,10 +2724,10 @@
       <c r="B40" s="20"/>
       <c r="C40" s="20"/>
       <c r="D40" s="20" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="E40" s="20" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
@@ -2732,10 +2735,10 @@
       <c r="B41" s="22"/>
       <c r="C41" s="22"/>
       <c r="D41" s="22" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
@@ -2743,10 +2746,10 @@
       <c r="B42" s="20"/>
       <c r="C42" s="20"/>
       <c r="D42" s="20" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="E42" s="20" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
@@ -2754,10 +2757,10 @@
       <c r="B43" s="22"/>
       <c r="C43" s="22"/>
       <c r="D43" s="22" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
@@ -2765,10 +2768,10 @@
       <c r="B44" s="20"/>
       <c r="C44" s="20"/>
       <c r="D44" s="20" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="E44" s="20" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
@@ -2776,10 +2779,10 @@
       <c r="B45" s="22"/>
       <c r="C45" s="22"/>
       <c r="D45" s="22" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
@@ -2787,10 +2790,10 @@
       <c r="B46" s="20"/>
       <c r="C46" s="20"/>
       <c r="D46" s="20" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="E46" s="20" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
@@ -2798,10 +2801,10 @@
       <c r="B47" s="22"/>
       <c r="C47" s="22"/>
       <c r="D47" s="22" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="E47" s="22" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
@@ -2809,10 +2812,10 @@
       <c r="B48" s="20"/>
       <c r="C48" s="20"/>
       <c r="D48" s="20" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="E48" s="20" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>
@@ -2844,20 +2847,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="51" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="49"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
+      <c r="K1" s="52"/>
+      <c r="L1" s="52"/>
     </row>
     <row r="2" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
@@ -2870,31 +2873,31 @@
         <v>2</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="M2" s="44"/>
       <c r="N2" s="44"/>
@@ -2911,19 +2914,19 @@
         <v>15</v>
       </c>
       <c r="D3" s="33" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="E3" s="20" t="s">
         <v>78</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="H3" s="20" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>30</v>
@@ -2943,10 +2946,10 @@
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="F4" s="17" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
@@ -2965,10 +2968,10 @@
       <c r="D5" s="20"/>
       <c r="E5" s="20"/>
       <c r="F5" s="20" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="H5" s="20"/>
       <c r="I5" s="20"/>
@@ -2987,10 +2990,10 @@
       <c r="D6" s="17"/>
       <c r="E6" s="17"/>
       <c r="F6" s="17" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="H6" s="17"/>
       <c r="I6" s="17"/>
@@ -3006,22 +3009,22 @@
         <v>64</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>78</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="G7" s="33" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="I7" s="20"/>
       <c r="J7" s="20"/>
@@ -3036,22 +3039,22 @@
         <v>65</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="E8" s="17" t="s">
         <v>78</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="I8" s="17"/>
       <c r="J8" s="17"/>
@@ -3069,10 +3072,10 @@
       <c r="D9" s="20"/>
       <c r="E9" s="20"/>
       <c r="F9" s="20" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="G9" s="33" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="H9" s="20"/>
       <c r="I9" s="20"/>
@@ -3088,19 +3091,19 @@
         <v>66</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>78</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
@@ -3116,10 +3119,10 @@
         <v>69</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="E11" s="20" t="s">
         <v>78</v>
@@ -3145,10 +3148,10 @@
       <c r="D12" s="17"/>
       <c r="E12" s="17"/>
       <c r="F12" s="17" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
@@ -3164,19 +3167,19 @@
         <v>67</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="E13" s="20" t="s">
         <v>78</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="G13" s="33" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="H13" s="20"/>
       <c r="I13" s="20" t="s">
@@ -3194,19 +3197,19 @@
         <v>70</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="E14" s="17" t="s">
         <v>78</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="H14" s="17"/>
       <c r="I14" s="17"/>
@@ -3225,10 +3228,10 @@
       <c r="D15" s="20"/>
       <c r="E15" s="20"/>
       <c r="F15" s="20" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="G15" s="33" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="H15" s="20"/>
       <c r="I15" s="20"/>
@@ -3238,19 +3241,19 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="17" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="D16" s="17"/>
       <c r="E16" s="17"/>
       <c r="F16" s="17"/>
       <c r="G16" s="17" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
@@ -3258,27 +3261,27 @@
         <v>14</v>
       </c>
       <c r="K16" s="17" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="L16" s="17" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="17" spans="1:12" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="20" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="B17" s="20" t="s">
+        <v>367</v>
+      </c>
+      <c r="C17" s="20" t="s">
         <v>372</v>
-      </c>
-      <c r="C17" s="20" t="s">
-        <v>377</v>
       </c>
       <c r="D17" s="20"/>
       <c r="E17" s="20"/>
       <c r="F17" s="20"/>
       <c r="G17" s="20" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="H17" s="20"/>
       <c r="I17" s="20"/>
@@ -3286,27 +3289,27 @@
         <v>14</v>
       </c>
       <c r="K17" s="20" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="L17" s="20" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="17" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="B18" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="C18" s="17" t="s">
         <v>373</v>
-      </c>
-      <c r="C18" s="17" t="s">
-        <v>378</v>
       </c>
       <c r="D18" s="17"/>
       <c r="E18" s="17"/>
       <c r="F18" s="17"/>
       <c r="G18" s="4" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
@@ -3314,27 +3317,27 @@
         <v>14</v>
       </c>
       <c r="K18" s="17" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="L18" s="17" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="19" spans="1:12" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="20" t="s">
+        <v>364</v>
+      </c>
+      <c r="B19" s="20" t="s">
         <v>369</v>
       </c>
-      <c r="B19" s="20" t="s">
-        <v>374</v>
-      </c>
       <c r="C19" s="20" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="D19" s="20"/>
       <c r="E19" s="20"/>
       <c r="F19" s="20"/>
       <c r="G19" s="20" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="H19" s="20"/>
       <c r="I19" s="20"/>
@@ -3342,27 +3345,27 @@
         <v>69</v>
       </c>
       <c r="K19" s="20" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="L19" s="20" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="17" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="B20" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="C20" s="17" t="s">
         <v>375</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>380</v>
       </c>
       <c r="D20" s="17"/>
       <c r="E20" s="17"/>
       <c r="F20" s="17"/>
       <c r="G20" s="17" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="H20" s="17"/>
       <c r="I20" s="17"/>
@@ -3370,27 +3373,27 @@
         <v>69</v>
       </c>
       <c r="K20" s="17" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="L20" s="17" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
     </row>
     <row r="21" spans="1:12" s="21" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A21" s="20" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="D21" s="20"/>
       <c r="E21" s="20"/>
       <c r="F21" s="20"/>
       <c r="G21" s="20" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="H21" s="20"/>
       <c r="I21" s="20"/>
@@ -3398,10 +3401,10 @@
         <v>69</v>
       </c>
       <c r="K21" s="20" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="L21" s="20" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
@@ -3412,12 +3415,12 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="F24" s="46" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="F25" s="46" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
     </row>
   </sheetData>
@@ -3442,14 +3445,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="51" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
@@ -3465,10 +3468,10 @@
         <v>63</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="G2" s="21"/>
     </row>
@@ -3480,13 +3483,13 @@
         <v>30</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D3" s="20" t="s">
         <v>73</v>
       </c>
       <c r="E3" s="33" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="F3" s="20" t="s">
         <v>78</v>
@@ -3498,34 +3501,34 @@
         <v>129</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>74</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="F4" s="5"/>
     </row>
     <row r="5" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="20" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B5" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="C5" s="33" t="s">
         <v>183</v>
-      </c>
-      <c r="C5" s="33" t="s">
-        <v>186</v>
       </c>
       <c r="D5" s="20" t="s">
         <v>74</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="F5" s="20"/>
     </row>
@@ -3534,16 +3537,16 @@
         <v>17</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D6" s="18" t="s">
         <v>73</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="F6" s="18"/>
     </row>
@@ -3555,13 +3558,13 @@
         <v>145</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>75</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="F7" s="12"/>
     </row>
@@ -3573,13 +3576,13 @@
         <v>146</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D8" s="18" t="s">
         <v>76</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="F8" s="18"/>
     </row>
@@ -3591,13 +3594,13 @@
         <v>147</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="F9" s="20"/>
     </row>
@@ -3609,13 +3612,13 @@
         <v>131</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D10" s="18" t="s">
         <v>73</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="F10" s="18"/>
     </row>
@@ -3642,15 +3645,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="51" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
@@ -3672,7 +3675,7 @@
         <v>158</v>
       </c>
       <c r="G2" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3683,7 +3686,7 @@
         <v>144</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>149</v>
@@ -3695,7 +3698,7 @@
         <v>23</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -3706,7 +3709,7 @@
         <v>152</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D4" s="31" t="s">
         <v>151</v>
@@ -3714,7 +3717,7 @@
       <c r="E4" s="31"/>
       <c r="F4" s="31"/>
       <c r="G4" s="31" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
@@ -3725,7 +3728,7 @@
         <v>154</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>155</v>
@@ -3735,7 +3738,7 @@
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
@@ -3743,37 +3746,37 @@
         <v>153</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C6" s="30" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="E6" s="30" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="F6" s="31"/>
       <c r="G6" s="31" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="33" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B7" s="20" t="s">
         <v>68</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D7" s="20"/>
       <c r="E7" s="20"/>
       <c r="F7" s="33"/>
       <c r="G7" s="33" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="H7" s="33"/>
     </row>
@@ -3782,56 +3785,56 @@
         <v>153</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C8" s="30" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="F8" s="30"/>
       <c r="G8" s="31" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="H8" s="33"/>
     </row>
     <row r="9" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="20" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B9" s="20" t="s">
         <v>134</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D9" s="20"/>
       <c r="E9" s="20"/>
       <c r="F9" s="20"/>
       <c r="G9" s="33" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="H9" s="20"/>
     </row>
     <row r="10" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="30" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B10" s="30" t="s">
         <v>142</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D10" s="30"/>
       <c r="E10" s="30"/>
       <c r="F10" s="30"/>
       <c r="G10" s="31" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="H10" s="20"/>
     </row>
@@ -3858,14 +3861,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="51" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
       <c r="G1" s="21"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -3885,7 +3888,7 @@
         <v>92</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="G2" s="16"/>
     </row>
@@ -3897,7 +3900,7 @@
         <v>78</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>139</v>
@@ -3914,7 +3917,7 @@
         <v>79</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D4" s="19" t="s">
         <v>84</v>
@@ -3931,7 +3934,7 @@
         <v>20</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>21</v>
@@ -3950,7 +3953,7 @@
         <v>80</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>85</v>
@@ -3967,10 +3970,10 @@
         <v>81</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -3984,10 +3987,10 @@
         <v>82</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
@@ -4001,7 +4004,7 @@
         <v>99</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>86</v>
@@ -4018,7 +4021,7 @@
         <v>83</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="D10" s="19" t="s">
         <v>87</v>
@@ -4073,7 +4076,7 @@
         <v>140</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D13" s="20" t="s">
         <v>21</v>
@@ -4093,7 +4096,7 @@
         <v>141</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>21</v>
@@ -4109,7 +4112,7 @@
         <v>89</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D15" s="20" t="s">
         <v>21</v>
@@ -4125,7 +4128,7 @@
         <v>90</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D16" s="19" t="s">
         <v>21</v>
@@ -4142,7 +4145,7 @@
         <v>91</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>88</v>
@@ -4152,38 +4155,30 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="19" t="s">
-        <v>161</v>
-      </c>
-      <c r="B18" s="19" t="s">
         <v>159</v>
       </c>
+      <c r="B18" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C18" s="19" t="s">
-        <v>213</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>14</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
       <c r="F18" s="19"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>160</v>
+        <v>425</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
     <row r="21" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.3"/>
@@ -4213,19 +4208,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-    </row>
-    <row r="2" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="53"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+    </row>
+    <row r="2" spans="1:9" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>72</v>
       </c>
@@ -4236,22 +4231,22 @@
         <v>2</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>249</v>
+        <v>426</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4262,7 +4257,7 @@
         <v>95</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D3" s="12"/>
       <c r="E3" s="2" t="s">
@@ -4274,7 +4269,7 @@
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4285,7 +4280,7 @@
         <v>96</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>95</v>
@@ -4294,16 +4289,16 @@
         <v>156</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="G4" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="H4" s="22" t="s">
-        <v>159</v>
+      <c r="H4" s="7" t="s">
+        <v>424</v>
       </c>
       <c r="I4" s="22" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4314,7 +4309,7 @@
         <v>97</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D5" s="20" t="s">
         <v>96</v>
@@ -4323,14 +4318,14 @@
         <v>14</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="G5" s="12" t="s">
         <v>80</v>
       </c>
       <c r="H5" s="12"/>
       <c r="I5" s="12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4341,7 +4336,7 @@
         <v>98</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D6" s="22" t="s">
         <v>97</v>
@@ -4355,7 +4350,7 @@
       </c>
       <c r="H6" s="22"/>
       <c r="I6" s="22" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4363,10 +4358,10 @@
         <v>120</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D7" s="20" t="s">
         <v>98</v>
@@ -4376,11 +4371,11 @@
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="12" t="s">
-        <v>160</v>
+      <c r="H7" s="2" t="s">
+        <v>425</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4391,23 +4386,23 @@
         <v>100</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>14</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="G8" s="22" t="s">
         <v>83</v>
       </c>
       <c r="H8" s="22"/>
       <c r="I8" s="22" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4418,7 +4413,7 @@
         <v>101</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D9" s="33" t="s">
         <v>100</v>
@@ -4432,7 +4427,7 @@
       </c>
       <c r="H9" s="12"/>
       <c r="I9" s="12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4440,10 +4435,10 @@
         <v>120</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D10" s="22" t="s">
         <v>101</v>
@@ -4459,7 +4454,7 @@
       </c>
       <c r="H10" s="22"/>
       <c r="I10" s="22" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4470,10 +4465,10 @@
         <v>102</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E11" s="12" t="s">
         <v>124</v>
@@ -4486,7 +4481,7 @@
       </c>
       <c r="H11" s="12"/>
       <c r="I11" s="12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4497,7 +4492,7 @@
         <v>103</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D12" s="22" t="s">
         <v>102</v>
@@ -4511,7 +4506,7 @@
       </c>
       <c r="H12" s="22"/>
       <c r="I12" s="22" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4522,7 +4517,7 @@
         <v>104</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D13" s="20" t="s">
         <v>103</v>
@@ -4536,7 +4531,7 @@
       </c>
       <c r="H13" s="12"/>
       <c r="I13" s="12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4547,7 +4542,7 @@
         <v>105</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D14" s="22" t="s">
         <v>104</v>
@@ -4559,7 +4554,7 @@
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
       <c r="I14" s="22" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="15" spans="1:9" s="9" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
@@ -4570,7 +4565,7 @@
         <v>132</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D15" s="20" t="s">
         <v>105</v>
@@ -4582,7 +4577,7 @@
       <c r="G15" s="12"/>
       <c r="H15" s="12"/>
       <c r="I15" s="12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4593,7 +4588,7 @@
         <v>106</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D16" s="22" t="s">
         <v>132</v>
@@ -4605,7 +4600,7 @@
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
       <c r="I16" s="22" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4616,7 +4611,7 @@
         <v>107</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D17" s="20" t="s">
         <v>106</v>
@@ -4630,7 +4625,7 @@
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="18" spans="1:9" s="9" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
@@ -4638,10 +4633,10 @@
         <v>120</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D18" s="22" t="s">
         <v>107</v>
@@ -4653,7 +4648,7 @@
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
       <c r="I18" s="22" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4664,10 +4659,10 @@
         <v>108</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>126</v>
@@ -4676,7 +4671,7 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4687,7 +4682,7 @@
         <v>109</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D20" s="22" t="s">
         <v>108</v>
@@ -4699,7 +4694,7 @@
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
       <c r="I20" s="22" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
@@ -4710,19 +4705,19 @@
         <v>110</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D21" s="20" t="s">
         <v>109</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
@@ -4752,14 +4747,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="51" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
@@ -4775,10 +4770,10 @@
         <v>127</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H2" s="9"/>
     </row>
@@ -4790,14 +4785,14 @@
         <v>27</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>95</v>
       </c>
       <c r="E3" s="23"/>
       <c r="F3" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G3" s="9"/>
       <c r="H3" s="9"/>
@@ -4810,14 +4805,14 @@
         <v>28</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>95</v>
       </c>
       <c r="E4" s="34"/>
       <c r="F4" s="8" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G4" s="9"/>
       <c r="H4" s="9"/>
@@ -4830,12 +4825,12 @@
         <v>29</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="23"/>
       <c r="F5" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G5" s="9"/>
       <c r="H5" s="9"/>
@@ -4848,12 +4843,12 @@
         <v>31</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D6" s="8"/>
       <c r="E6" s="34"/>
       <c r="F6" s="8" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G6" s="9"/>
     </row>
@@ -4865,16 +4860,16 @@
         <v>32</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>96</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G7" s="9"/>
     </row>
@@ -4886,16 +4881,16 @@
         <v>33</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D8" s="24" t="s">
         <v>97</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G8" s="9"/>
     </row>
@@ -4907,14 +4902,14 @@
         <v>34</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>98</v>
       </c>
       <c r="E9" s="23"/>
       <c r="F9" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G9" s="9"/>
     </row>
@@ -4926,16 +4921,16 @@
         <v>35</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G10" s="9"/>
     </row>
@@ -4947,16 +4942,16 @@
         <v>36</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>100</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G11" s="9"/>
     </row>
@@ -4968,16 +4963,16 @@
         <v>37</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>100</v>
       </c>
       <c r="E12" s="24" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G12" s="9"/>
     </row>
@@ -4989,14 +4984,14 @@
         <v>38</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>101</v>
       </c>
       <c r="E13" s="23"/>
       <c r="F13" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G13" s="9"/>
     </row>
@@ -5008,14 +5003,14 @@
         <v>39</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D14" s="24" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E14" s="34"/>
       <c r="F14" s="8" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G14" s="9"/>
     </row>
@@ -5027,14 +5022,14 @@
         <v>40</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="D15" s="12" t="s">
         <v>102</v>
       </c>
       <c r="E15" s="23"/>
       <c r="F15" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G15" s="9"/>
     </row>
@@ -5046,14 +5041,14 @@
         <v>41</v>
       </c>
       <c r="C16" s="24" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>102</v>
       </c>
       <c r="E16" s="34"/>
       <c r="F16" s="8" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G16" s="9"/>
     </row>
@@ -5065,14 +5060,14 @@
         <v>42</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>103</v>
       </c>
       <c r="E17" s="23"/>
       <c r="F17" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G17" s="9"/>
     </row>
@@ -5084,14 +5079,14 @@
         <v>43</v>
       </c>
       <c r="C18" s="24" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>104</v>
       </c>
       <c r="E18" s="34"/>
       <c r="F18" s="8" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G18" s="9"/>
     </row>
@@ -5103,14 +5098,14 @@
         <v>44</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>105</v>
       </c>
       <c r="E19" s="23"/>
       <c r="F19" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G19" s="9"/>
     </row>
@@ -5122,14 +5117,14 @@
         <v>45</v>
       </c>
       <c r="C20" s="24" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>106</v>
       </c>
       <c r="E20" s="34"/>
       <c r="F20" s="8" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G20" s="9"/>
     </row>
@@ -5141,14 +5136,14 @@
         <v>46</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="D21" s="12" t="s">
         <v>107</v>
       </c>
       <c r="E21" s="35"/>
       <c r="F21" s="43" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -5159,14 +5154,14 @@
         <v>47</v>
       </c>
       <c r="C22" s="24" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D22" s="24" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="E22" s="34"/>
       <c r="F22" s="8" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G22" s="9"/>
     </row>
@@ -5178,16 +5173,16 @@
         <v>48</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D23" s="12" t="s">
         <v>108</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G23" s="9"/>
     </row>
@@ -5199,14 +5194,14 @@
         <v>49</v>
       </c>
       <c r="C24" s="24" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="D24" s="24" t="s">
         <v>109</v>
       </c>
       <c r="E24" s="34"/>
       <c r="F24" s="8" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G24" s="9"/>
     </row>
@@ -5218,14 +5213,14 @@
         <v>128</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="D25" s="12" t="s">
         <v>110</v>
       </c>
       <c r="E25" s="12"/>
       <c r="F25" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="G25" s="9"/>
     </row>
@@ -5285,7 +5280,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -5293,22 +5288,24 @@
     <col min="3" max="3" width="35" customWidth="1"/>
     <col min="4" max="4" width="26.109375" customWidth="1"/>
     <col min="5" max="7" width="26.109375" style="47" customWidth="1"/>
-    <col min="8" max="8" width="39" customWidth="1"/>
+    <col min="8" max="8" width="21" style="48" customWidth="1"/>
+    <col min="9" max="9" width="39" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="51" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-    </row>
-    <row r="2" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+    </row>
+    <row r="2" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>72</v>
       </c>
@@ -5319,36 +5316,39 @@
         <v>2</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>400</v>
-      </c>
-      <c r="F2" s="10" t="s">
+        <v>395</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="20" t="s">
+        <v>391</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>393</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>410</v>
+      </c>
+      <c r="D3" s="20" t="s">
         <v>399</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="20" t="s">
-        <v>396</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>398</v>
-      </c>
-      <c r="C3" s="20" t="s">
-        <v>415</v>
-      </c>
-      <c r="D3" s="20" t="s">
-        <v>404</v>
-      </c>
       <c r="E3" s="20" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="F3" s="20" t="s">
         <v>14</v>
@@ -5357,46 +5357,48 @@
         <v>95</v>
       </c>
       <c r="H3" s="20"/>
-    </row>
-    <row r="4" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="52" t="s">
-        <v>396</v>
-      </c>
-      <c r="B4" s="52" t="s">
-        <v>403</v>
-      </c>
-      <c r="C4" s="52" t="s">
-        <v>416</v>
-      </c>
-      <c r="D4" s="52" t="s">
-        <v>404</v>
-      </c>
-      <c r="E4" s="52" t="s">
-        <v>402</v>
-      </c>
-      <c r="F4" s="52" t="s">
+      <c r="I3" s="20"/>
+    </row>
+    <row r="4" spans="1:9" s="21" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="50" t="s">
+        <v>391</v>
+      </c>
+      <c r="B4" s="50" t="s">
+        <v>398</v>
+      </c>
+      <c r="C4" s="50" t="s">
+        <v>411</v>
+      </c>
+      <c r="D4" s="50" t="s">
+        <v>399</v>
+      </c>
+      <c r="E4" s="50" t="s">
+        <v>397</v>
+      </c>
+      <c r="F4" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="G4" s="52" t="s">
+      <c r="G4" s="50" t="s">
         <v>95</v>
       </c>
-      <c r="H4" s="52"/>
-    </row>
-    <row r="5" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="H4" s="50"/>
+      <c r="I4" s="50"/>
+    </row>
+    <row r="5" spans="1:9" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="20" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="B5" s="20" t="s">
+        <v>407</v>
+      </c>
+      <c r="C5" s="20" t="s">
         <v>412</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>417</v>
       </c>
       <c r="D5" s="20" t="s">
         <v>135</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="F5" s="20" t="s">
         <v>14</v>
@@ -5405,94 +5407,98 @@
         <v>108</v>
       </c>
       <c r="H5" s="20"/>
-    </row>
-    <row r="6" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="52" t="s">
-        <v>396</v>
-      </c>
-      <c r="B6" s="52" t="s">
-        <v>411</v>
-      </c>
-      <c r="C6" s="52" t="s">
-        <v>418</v>
-      </c>
-      <c r="D6" s="52" t="s">
+      <c r="I5" s="20"/>
+    </row>
+    <row r="6" spans="1:9" s="21" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="50" t="s">
+        <v>391</v>
+      </c>
+      <c r="B6" s="50" t="s">
+        <v>406</v>
+      </c>
+      <c r="C6" s="50" t="s">
+        <v>413</v>
+      </c>
+      <c r="D6" s="50" t="s">
         <v>135</v>
       </c>
-      <c r="E6" s="52" t="s">
-        <v>413</v>
-      </c>
-      <c r="F6" s="52" t="s">
+      <c r="E6" s="50" t="s">
+        <v>408</v>
+      </c>
+      <c r="F6" s="50" t="s">
         <v>65</v>
       </c>
-      <c r="G6" s="52" t="s">
+      <c r="G6" s="50" t="s">
         <v>108</v>
       </c>
-      <c r="H6" s="52"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H6" s="50"/>
+      <c r="I6" s="50"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="20" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="F7" s="20" t="s">
         <v>65</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="H7" s="20"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="52" t="s">
-        <v>396</v>
-      </c>
-      <c r="B8" s="52" t="s">
-        <v>407</v>
-      </c>
-      <c r="C8" s="52" t="s">
-        <v>420</v>
-      </c>
-      <c r="D8" s="52" t="s">
+      <c r="I7" s="20"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="50" t="s">
+        <v>391</v>
+      </c>
+      <c r="B8" s="50" t="s">
+        <v>402</v>
+      </c>
+      <c r="C8" s="50" t="s">
+        <v>415</v>
+      </c>
+      <c r="D8" s="50" t="s">
+        <v>400</v>
+      </c>
+      <c r="E8" s="50" t="s">
+        <v>397</v>
+      </c>
+      <c r="F8" s="50" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8" s="50" t="s">
+        <v>261</v>
+      </c>
+      <c r="H8" s="50"/>
+      <c r="I8" s="50"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
+        <v>391</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>403</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>416</v>
+      </c>
+      <c r="D9" s="20" t="s">
         <v>405</v>
       </c>
-      <c r="E8" s="52" t="s">
-        <v>402</v>
-      </c>
-      <c r="F8" s="52" t="s">
-        <v>66</v>
-      </c>
-      <c r="G8" s="52" t="s">
-        <v>265</v>
-      </c>
-      <c r="H8" s="52"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="20" t="s">
-        <v>396</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>408</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>421</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>410</v>
-      </c>
       <c r="E9" s="20" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="F9" s="20" t="s">
         <v>65</v>
@@ -5501,96 +5507,101 @@
         <v>109</v>
       </c>
       <c r="H9" s="20"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="52" t="s">
-        <v>396</v>
-      </c>
-      <c r="B10" s="52" t="s">
-        <v>409</v>
-      </c>
-      <c r="C10" s="52" t="s">
-        <v>422</v>
-      </c>
-      <c r="D10" s="52" t="s">
-        <v>410</v>
-      </c>
-      <c r="E10" s="52" t="s">
-        <v>397</v>
-      </c>
-      <c r="F10" s="52" t="s">
+      <c r="I9" s="20"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" s="50" t="s">
+        <v>391</v>
+      </c>
+      <c r="B10" s="50" t="s">
+        <v>404</v>
+      </c>
+      <c r="C10" s="50" t="s">
+        <v>417</v>
+      </c>
+      <c r="D10" s="50" t="s">
+        <v>405</v>
+      </c>
+      <c r="E10" s="50" t="s">
+        <v>392</v>
+      </c>
+      <c r="F10" s="50" t="s">
         <v>70</v>
       </c>
-      <c r="G10" s="52" t="s">
+      <c r="G10" s="50" t="s">
         <v>109</v>
       </c>
-      <c r="H10" s="52"/>
-    </row>
-    <row r="11" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="H10" s="50"/>
+      <c r="I10" s="50"/>
+    </row>
+    <row r="11" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="20" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="G11" s="33" t="s">
         <v>105</v>
       </c>
-      <c r="H11" s="20"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="52" t="s">
+      <c r="H11" s="33"/>
+      <c r="I11" s="20"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="50" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="52" t="s">
-        <v>330</v>
-      </c>
-      <c r="C12" s="52" t="s">
-        <v>328</v>
-      </c>
-      <c r="D12" s="52" t="s">
+      <c r="B12" s="50" t="s">
+        <v>326</v>
+      </c>
+      <c r="C12" s="50" t="s">
+        <v>324</v>
+      </c>
+      <c r="D12" s="50"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="50"/>
+      <c r="G12" s="50"/>
+      <c r="H12" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="52"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="52"/>
-      <c r="H12" s="52" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="I12" s="50" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="20" t="s">
         <v>50</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>329</v>
-      </c>
-      <c r="D13" s="20" t="s">
-        <v>65</v>
-      </c>
+        <v>325</v>
+      </c>
+      <c r="D13" s="20"/>
       <c r="E13" s="20"/>
       <c r="F13" s="20"/>
       <c r="G13" s="20"/>
-      <c r="H13" s="20" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H13" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="I13" s="33" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="21"/>
       <c r="B14" s="21"/>
       <c r="C14" s="21"/>
@@ -5598,55 +5609,56 @@
       <c r="E14" s="21"/>
       <c r="F14" s="21"/>
       <c r="G14" s="21"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H14" s="21"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E15"/>
       <c r="F15"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="38"/>
       <c r="E16"/>
       <c r="F16"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="51"/>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="49"/>
       <c r="E17"/>
       <c r="F17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="51"/>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="49"/>
       <c r="E18"/>
       <c r="F18"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="51"/>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="49"/>
       <c r="C19" s="47"/>
       <c r="E19"/>
       <c r="F19"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C20" s="47"/>
       <c r="E20"/>
       <c r="F20"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C21" s="47"/>
       <c r="E21"/>
       <c r="F21"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C22" s="47"/>
       <c r="D22" s="47"/>
       <c r="E22"/>
       <c r="F22"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C23" s="47"/>
       <c r="D23" s="47"/>
       <c r="E23"/>
       <c r="F23"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="29"/>
       <c r="B27" s="29"/>
       <c r="C27" s="29"/>
@@ -5654,34 +5666,39 @@
       <c r="E27" s="29"/>
       <c r="F27" s="29"/>
       <c r="G27" s="29"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H27" s="29"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D28" s="40"/>
       <c r="E28" s="40"/>
       <c r="F28" s="40"/>
       <c r="G28" s="40"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H28" s="40"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D31" s="40"/>
       <c r="E31" s="40"/>
       <c r="F31" s="40"/>
       <c r="G31" s="40"/>
-    </row>
-    <row r="33" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="H31" s="40"/>
+    </row>
+    <row r="33" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D33" s="40"/>
       <c r="E33" s="40"/>
       <c r="F33" s="40"/>
       <c r="G33" s="40"/>
-    </row>
-    <row r="34" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="H33" s="40"/>
+    </row>
+    <row r="34" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D34" s="40"/>
       <c r="E34" s="40"/>
       <c r="F34" s="40"/>
       <c r="G34" s="40"/>
+      <c r="H34" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5699,12 +5716,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="51" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
     </row>
     <row r="2" spans="1:4" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
@@ -5717,7 +5734,7 @@
         <v>2</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -5728,7 +5745,7 @@
         <v>115</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>14</v>
@@ -5742,7 +5759,7 @@
         <v>116</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D4" s="19" t="s">
         <v>14</v>
@@ -5756,7 +5773,7 @@
         <v>117</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>14</v>
@@ -5767,10 +5784,10 @@
         <v>52</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>100</v>
@@ -5781,10 +5798,10 @@
         <v>52</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>110</v>
@@ -5795,10 +5812,10 @@
         <v>52</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D8" s="19" t="s">
         <v>97</v>
@@ -5809,13 +5826,13 @@
         <v>52</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>